<commit_message>
files update for bulk upload
</commit_message>
<xml_diff>
--- a/public/sampleFiles/case_sample_file.xlsx
+++ b/public/sampleFiles/case_sample_file.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\ThirdEx\sample files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Thirdex\thirdxui\public\sampleFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C792B9E-8B28-4727-8707-A7C4D0496BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>service_user</t>
   </si>
@@ -41,39 +42,6 @@
     <t>case_closed_date</t>
   </si>
   <si>
-    <t>engagement</t>
-  </si>
-  <si>
-    <t>demo, deo</t>
-  </si>
-  <si>
-    <t>campaigns one, campaigns two</t>
-  </si>
-  <si>
-    <t>Engagement two, Engagement one</t>
-  </si>
-  <si>
-    <t>event two, event one</t>
-  </si>
-  <si>
-    <t>funding two</t>
-  </si>
-  <si>
-    <t>benificiary_information</t>
-  </si>
-  <si>
-    <t>campaigns_supported</t>
-  </si>
-  <si>
-    <t>events_attended</t>
-  </si>
-  <si>
-    <t>funding_interests</t>
-  </si>
-  <si>
-    <t>fundraising_activities</t>
-  </si>
-  <si>
     <t>notes</t>
   </si>
   <si>
@@ -93,12 +61,18 @@
   </si>
   <si>
     <t>uploads/file-1749463679399.jpg</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>emp1, hindu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -413,26 +387,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="1" max="1" width="16.81640625" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" customWidth="1"/>
-    <col min="8" max="8" width="24.33203125" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" customWidth="1"/>
-    <col min="11" max="11" width="18.33203125" customWidth="1"/>
-    <col min="12" max="12" width="17.33203125" customWidth="1"/>
-    <col min="13" max="13" width="16.77734375" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="18.36328125" customWidth="1"/>
+    <col min="6" max="6" width="21.6328125" customWidth="1"/>
+    <col min="7" max="7" width="17.36328125" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -449,39 +418,24 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2">
         <v>45846</v>
@@ -490,28 +444,13 @@
         <v>45854</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>